<commit_message>
V9 F5: salidas regeneradas (publicacion, base con v9_efectos, consulta, web_resumen)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GDwCFFTud391ebBMaJpdsw
</commit_message>
<xml_diff>
--- a/publicacion/tablas_v9.xlsx
+++ b/publicacion/tablas_v9.xlsx
@@ -1368,7 +1368,7 @@
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="D19" s="3" t="n"/>
       <c r="E19" s="3" t="n"/>
@@ -2591,7 +2591,7 @@
         </is>
       </c>
       <c r="C44" s="3" t="n">
-        <v>2215895</v>
+        <v>2177711</v>
       </c>
       <c r="D44" s="3" t="n"/>
       <c r="E44" s="3" t="n"/>
@@ -2732,7 +2732,7 @@
         </is>
       </c>
       <c r="C47" s="3" t="n">
-        <v>84.43304032</v>
+        <v>111.6309578</v>
       </c>
       <c r="D47" s="3" t="n"/>
       <c r="E47" s="3" t="n"/>
@@ -2779,7 +2779,7 @@
         </is>
       </c>
       <c r="C48" s="3" t="n">
-        <v>152576</v>
+        <v>114392</v>
       </c>
       <c r="D48" s="3" t="n"/>
       <c r="E48" s="3" t="n"/>
@@ -3155,7 +3155,7 @@
         </is>
       </c>
       <c r="C56" s="3" t="n">
-        <v>19762059</v>
+        <v>19521046</v>
       </c>
       <c r="D56" s="3" t="n"/>
       <c r="E56" s="3" t="n"/>
@@ -3296,7 +3296,7 @@
         </is>
       </c>
       <c r="C59" s="3" t="n">
-        <v>68.85463129</v>
+        <v>91.96270552999999</v>
       </c>
       <c r="D59" s="3" t="n"/>
       <c r="E59" s="3" t="n"/>
@@ -3343,7 +3343,7 @@
         </is>
       </c>
       <c r="C60" s="3" t="n">
-        <v>939956</v>
+        <v>698943</v>
       </c>
       <c r="D60" s="3" t="n"/>
       <c r="E60" s="3" t="n"/>

</xml_diff>